<commit_message>
completed divisibilty & primes
</commit_message>
<xml_diff>
--- a/Middle_School_Olympiad_Platform_BIDMAS.xlsx
+++ b/Middle_School_Olympiad_Platform_BIDMAS.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,12 @@
       <color theme="10"/>
       <sz val="11"/>
       <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <sz val="8"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -442,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3577,6 +3583,1286 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>AMC 8</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/amc-div-question1.png</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/amc-div-answer1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>AMC 8</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/amc-div-question2.png</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/amc-div-answer2.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>AMC 8</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/amc-div-question3.png</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/amc-div-answer3.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>AMC 8</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/amc-div-question4.png</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/amc-div-answer4.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-question1.png</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-answer1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-question2.png</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-answer2.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-question3.png</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-answer3.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-question4.png</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-answer4.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-question5.png</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-answer5.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-question6.png</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-answer6.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-question7.png</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-answer7.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-question8.png</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-answer8.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-question9.png</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-answer9.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-question10.png</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-answer10.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-question11.png</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-answer11.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-question1.png</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-answer1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-question2.png</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-answer2.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-question3.png</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-answer3.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-question4.png</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-answer4.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-question5.png</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-answer5.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-question6.png</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-answer6.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-question7.png</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-answer7.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-question8.png</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-answer8.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-question9.png</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/ukmt-jmc-prime-prop-answer9.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>NMTC Primary</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-pri-question1.png</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-pri-answer1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>NMTC Primary</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-pri-question2.png</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-pri-answer2.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>NMTC Primary</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-pri-question3.png</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-pri-answer3.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>NMTC Primary</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-pri-question4.png</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-pri-answer4.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>NMTC Primary</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-pri-question5.png</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-pri-answer5.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>NMTC Sub Junior</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-question1.png</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-answer1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>NMTC Sub Junior</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-question2.png</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-answer2.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>NMTC Sub Junior</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-question3.png</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-answer3.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>NMTC Sub Junior</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-question4.png</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-answer4.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>NMTC Sub Junior</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-question5.png</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-answer5.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>NMTC Sub Junior</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-question6.png</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-answer6.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>NMTC Sub Junior</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-question7.png</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-answer7.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>NMTC Sub Junior</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Prime Properties</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-question8.png</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/nmtc-sub-answer8.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Math Count</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/m-count-question1.png</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/m-count-answer1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Math Count</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/m-count-question2.png</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/m-count-answer2.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Math Count</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Divisibility &amp; Primes</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Divisibility Rules</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/m-count-question3.png</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/divisibility-primes/refs/heads/main/m-count-answer3.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId1"/>

</xml_diff>

<commit_message>
completed modular thinking intro
</commit_message>
<xml_diff>
--- a/Middle_School_Olympiad_Platform_BIDMAS.xlsx
+++ b/Middle_School_Olympiad_Platform_BIDMAS.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L148"/>
+  <dimension ref="A1:L162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5375,6 +5375,454 @@
         </is>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>AMC 8</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Remainders</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/amc-question1.png</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/amc-answer1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>AMC 8</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Basic Modular Arithmetic</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/amc-question2.png</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/amc-answer2.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>AMC 8</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Basic Modular Arithmetic</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/amc-question3.png</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/amc-answer3.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Remainders</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/ukmt-jmc-question1.png</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/ukmt-jmc-answer1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Remainders</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/ukmt-jmc-question2.png</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/ukmt-jmc-answer2.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Remainders</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/ukmt-jmc-question3.png</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/ukmt-jmc-answer3.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>UKMT JMC</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Basic Modular Arithmetic</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/ukmt-jmc-question4.png</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/ukmt-jmc-answer4.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Math Count</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Remainders</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/math-count-question1.png</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/math-count-answer1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>NMTC Primary</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Remainders</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/nmtc-pri-question1.png</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/nmtc-pri-answer1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>NMTC Primary</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Remainders</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/nmtc-pri-question2.png</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/nmtc-pri-answer2.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>NMTC Primary</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Remainders</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/nmtc-pri-question3.png</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/nmtc-pri-answer3.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>NMTC Primary</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Remainders</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/nmtc-pri-question4.png</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/nmtc-pri-answer4.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>NMTC Primary</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Basic Modular Arithmetic</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/nmtc-pri-question5.png</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/nmtc-pri-answer5.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>NMTC Primary</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Modular Thinking (Intro)</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Basic Modular Arithmetic</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/nmtc-pri-question6.png</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Lalitha-Kalle/modular-thinking/refs/heads/main/nmtc-pri-answer6.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId1"/>

</xml_diff>